<commit_message>
Actualizar evidencias de Trello y GitHub
</commit_message>
<xml_diff>
--- a/Miga_y_Miel_Seguimiento_Nuevo_Enlace.xlsx
+++ b/Miga_y_Miel_Seguimiento_Nuevo_Enlace.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pan_c\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ed6d5ad3be95f9d/Documentos/Archivos Visual Studio Code/miga-miel-pasteleria/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EBB1F5B-6D4F-4222-B06F-16776A3D60D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{8EBB1F5B-6D4F-4222-B06F-16776A3D60D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05B2779E-E0EF-495F-89B9-8DCF78A1BA80}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="146">
   <si>
     <t>MIGA &amp; MIEL  |  HERRAMIENTAS DE SEGUIMIENTO</t>
   </si>
@@ -375,9 +375,6 @@
     <t>https://github.com</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Crear repositorio</t>
   </si>
   <si>
@@ -469,6 +466,15 @@
   </si>
   <si>
     <t>Completado</t>
+  </si>
+  <si>
+    <t>https://github.com/FranSpiller/miga-miel-pasteleria</t>
+  </si>
+  <si>
+    <t>https://trello.com/invite/b/6ae2f8dbe5af408ca41e1b58/ATTI28579f58c1dc2f9f3768d5bd0432e3b0EE29014A/miga-miel-proyecto-de-software</t>
+  </si>
+  <si>
+    <t>Trello URL:</t>
   </si>
 </sst>
 </file>
@@ -478,7 +484,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -527,6 +533,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF362F33"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -587,10 +599,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -617,22 +630,25 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
@@ -974,6 +990,99 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>525691</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>29544</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9536C05C-9278-50B9-A631-4E0D7DA58C6D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="847725" y="5981700"/>
+          <a:ext cx="13012966" cy="6944694"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>518407</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>35544</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4607583F-D60F-8177-B71B-E97F79870C0B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="840441" y="13032441"/>
+          <a:ext cx="13012966" cy="5772956"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
@@ -1191,15 +1300,15 @@
       <c r="G1" s="11"/>
     </row>
     <row r="2" spans="1:7" ht="29.1" customHeight="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="4" spans="1:7" ht="27.95" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -1283,94 +1392,94 @@
       <c r="G10" s="13"/>
     </row>
     <row r="11" spans="1:7" ht="27" customHeight="1">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
     </row>
     <row r="12" spans="1:7" ht="27" customHeight="1">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
     </row>
     <row r="13" spans="1:7" ht="27" customHeight="1">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
     </row>
     <row r="14" spans="1:7" ht="27" customHeight="1">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
     </row>
     <row r="15" spans="1:7" ht="27" customHeight="1">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
     </row>
     <row r="16" spans="1:7" ht="27" customHeight="1">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
     </row>
     <row r="18" spans="1:7" ht="30" customHeight="1">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1405,17 +1514,17 @@
       <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" ht="26.1" customHeight="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="4" spans="1:9" ht="24" customHeight="1">
       <c r="A4" s="3" t="s">
@@ -1470,7 +1579,7 @@
         <v>40</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>42</v>
@@ -1502,10 +1611,10 @@
         <v>49</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>50</v>
@@ -1529,10 +1638,10 @@
         <v>49</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>46</v>
@@ -1556,10 +1665,10 @@
         <v>49</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>51</v>
@@ -1583,10 +1692,10 @@
         <v>57</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>53</v>
@@ -1610,10 +1719,10 @@
         <v>57</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>46</v>
@@ -1637,10 +1746,10 @@
         <v>57</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>58</v>
@@ -1664,10 +1773,10 @@
         <v>64</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>65</v>
@@ -1691,10 +1800,10 @@
         <v>64</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>68</v>
@@ -1718,10 +1827,10 @@
         <v>71</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>66</v>
@@ -1745,10 +1854,10 @@
         <v>71</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>74</v>
@@ -1772,10 +1881,10 @@
         <v>64</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>53</v>
@@ -1799,10 +1908,10 @@
         <v>71</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>80</v>
@@ -1870,14 +1979,14 @@
       <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:9" ht="27.95" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
     </row>
     <row r="4" spans="1:9" ht="27.95" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -1890,7 +1999,7 @@
         <v>86</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>87</v>
@@ -1910,19 +2019,19 @@
         <v>46311</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>130</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>91</v>
@@ -1937,19 +2046,19 @@
         <v>46316</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>130</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>92</v>
@@ -1967,16 +2076,16 @@
         <v>49</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>93</v>
@@ -2197,7 +2306,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1">
       <c r="A1" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2208,16 +2317,16 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
     </row>
     <row r="4" spans="1:8" ht="27.95" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -2288,7 +2397,7 @@
         <v>46324</v>
       </c>
       <c r="C10" s="9">
-        <f t="shared" ref="C9:C16" si="0">MAX(0,$A$5*(1-A10/$B$5))</f>
+        <f t="shared" ref="C10:C15" si="0">MAX(0,$A$5*(1-A10/$B$5))</f>
         <v>37.5</v>
       </c>
       <c r="D10" s="10">
@@ -2368,12 +2477,12 @@
     </row>
     <row r="17" spans="1:4" ht="27" customHeight="1"/>
     <row r="19" spans="1:4" ht="30" customHeight="1">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2410,14 +2519,14 @@
       <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:6" ht="27.95" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
     </row>
     <row r="4" spans="1:6" ht="27.95" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -2430,7 +2539,7 @@
         <v>109</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27" customHeight="1">
@@ -2444,7 +2553,7 @@
         <v>111</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="27" customHeight="1">
@@ -2452,13 +2561,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>114</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="27" customHeight="1">
@@ -2466,13 +2575,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="27" customHeight="1">
@@ -2480,13 +2589,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>118</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="27" customHeight="1">
@@ -2494,13 +2603,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>120</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>112</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="27" customHeight="1">
@@ -2508,13 +2617,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="27" customHeight="1">
@@ -2522,13 +2631,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>124</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>112</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="27" customHeight="1">
@@ -2536,18 +2645,18 @@
         <v>8</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>126</v>
-      </c>
       <c r="D12" s="2" t="s">
-        <v>112</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="24" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
@@ -2556,22 +2665,32 @@
       <c r="F15" s="13"/>
     </row>
     <row r="16" spans="1:6" ht="33.950000000000003" customHeight="1">
-      <c r="A16" s="18"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
+      <c r="A16" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+    </row>
+    <row r="17" spans="1:6" ht="30.75" customHeight="1">
+      <c r="A17" t="s">
+        <v>145</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="18" spans="1:6" ht="38.1" customHeight="1">
-      <c r="A18" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
+      <c r="A18" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2586,6 +2705,11 @@
       <formula1>"No,Sí"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="A16" r:id="rId1" xr:uid="{31035573-B348-46EF-B06E-EEB4F65B5325}"/>
+    <hyperlink ref="B17" r:id="rId2" xr:uid="{708ECF5B-BCE1-4CFA-851D-9A21BA7231DF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>